<commit_message>
Implementação da visão de performance 1.0
</commit_message>
<xml_diff>
--- a/dimensoes.xlsx
+++ b/dimensoes.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PHONE STORE\Documents\PROJETIN_DOS_CRIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C886C412-F417-4CDA-8CCF-40D0B8771055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F834F210-446C-4C51-830A-8236638BEDB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{671B69D3-1FBE-4114-A181-B969F0E7BB39}"/>
   </bookViews>
   <sheets>
     <sheet name="Lojas" sheetId="1" r:id="rId1"/>
-    <sheet name="Regiões" sheetId="5" r:id="rId2"/>
-    <sheet name="Vendedores" sheetId="2" r:id="rId3"/>
-    <sheet name="Planos" sheetId="3" r:id="rId4"/>
-    <sheet name="Categorias" sheetId="4" r:id="rId5"/>
+    <sheet name="Dim_produtos" sheetId="6" r:id="rId2"/>
+    <sheet name="Regiões" sheetId="5" r:id="rId3"/>
+    <sheet name="Vendedores" sheetId="2" r:id="rId4"/>
+    <sheet name="Planos" sheetId="3" r:id="rId5"/>
+    <sheet name="Categorias" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1272" uniqueCount="979">
   <si>
     <t>V001</t>
   </si>
@@ -1727,12 +1728,1263 @@
   </si>
   <si>
     <t>PS - SHOP DA ILHA SLZ</t>
+  </si>
+  <si>
+    <t>PRODUTO</t>
+  </si>
+  <si>
+    <t>PREÇO</t>
+  </si>
+  <si>
+    <t>INFINIX SMART 10 128GB/4+4RAM - IRIS BLUE (1422)</t>
+  </si>
+  <si>
+    <t>INFINIX SMART 10 64GB/3+3RAM - TITANIUM SILVER (10000035)</t>
+  </si>
+  <si>
+    <t>ASUS ZENFONE MAX PRO 64GB - TITANIUM (538)</t>
+  </si>
+  <si>
+    <t>CELULAR BARRINHA ZTE PRETO (10000071)</t>
+  </si>
+  <si>
+    <t>CELULAR POSITIVO P26 - PRETO (1145)</t>
+  </si>
+  <si>
+    <t>CELULAR POSITIVO P26 - PRETO (923)</t>
+  </si>
+  <si>
+    <t>CELULAR POSITIVO P26 4G DUAL CHIP - PRETO (10000044)</t>
+  </si>
+  <si>
+    <t>CELULAR POSITIVO P41 DUAL CHIP 4G - PRETO (1144)</t>
+  </si>
+  <si>
+    <t>CELULAR TCL 605 128GB 4+8GGB RAM NFC - AZUL (10000032)</t>
+  </si>
+  <si>
+    <t>FIRE 6 256GB/16RAM- BLACK (10000083)</t>
+  </si>
+  <si>
+    <t>FONE BLUETOOTH APPLE EARPODS PRO 2 (791)</t>
+  </si>
+  <si>
+    <t>HONOR MAGIC 7 LITE - TITANIUM BLACK (1421)</t>
+  </si>
+  <si>
+    <t>HONOR PLAY 9A 128GB/4RAM - OCEAN BLUE (10000081)</t>
+  </si>
+  <si>
+    <t>HONOR X5B 128GB/4RAM - Negro Medianoche (10000046)</t>
+  </si>
+  <si>
+    <t>HONOR X5B 128GB/4RAM - NEGRO MEDIANOCHE (1057)</t>
+  </si>
+  <si>
+    <t>HONOR X5B 128GB/4RAM - OCEAN BLUE (1420)</t>
+  </si>
+  <si>
+    <t>HONOR X5B PLUS 256GB/4RAM - MIDNIGHT BLACK (1472)</t>
+  </si>
+  <si>
+    <t>HONOR X5B PLUS 256GB/4RAM - OCEAN BLUE (1473)</t>
+  </si>
+  <si>
+    <t>HONOR X6B 256GB/4RAM - NEGRO (10000079)</t>
+  </si>
+  <si>
+    <t>HONOR X7d 256GB/8RAM - PLATA METEORO (10000080)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 40 PRO 256GB / 16GB - STARFALL GREEN (1120)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 50 256GB/8+8RAM - SAGE GREEN (1262)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 50 256GB/8+8RAM - SLEEK BLACK (1261)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 50 256GB/8+8RAM - TITANIUM GREY (1263)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 50i 256GB/8+8RAM - SLEEK BLACK (10000075)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 50i 256GB/8+8RAM - TITANIUM GREY (10000076)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 60 PRO+ 256GB/16RAM - SLEEK BLACK (10000075)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 60I 256GB/4+4RAM - MEADOW GREEN (1428)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 60I 256GB/8+8RAM - SOUL EYE PURPLE (10000277)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 60I 256GB/8+8RAM - TITANIUM SILVER (1501)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 60I 256GB/4+4RAM - SLEEK BLACK (1439)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 60I 256GB/8+8RAM - MEADOW GREEN (1498)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 60I 256GB/8+8RAM - MEADOW GREEN (10000278)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 60I 256GB/8+8RAM - SOUL EYE PURPLE (1500)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 60I 256GB/8+8RAM - SLEEK BLACK (1521)</t>
+  </si>
+  <si>
+    <t>INFINIX SMART 10 128GB/4+4RAM - SLEEK BLACK (1390)</t>
+  </si>
+  <si>
+    <t>INFINIX SMART 10 128GB/4+4RAM - TITANIUM SILVER (10000282)</t>
+  </si>
+  <si>
+    <t>INFINIX SMART 10 128GB/4+4RAM - TITANIUM SILVER (1384)</t>
+  </si>
+  <si>
+    <t>INFINIX SMART 10 128GB/4+4RAM - TWILIGHT GOLD (10000281)</t>
+  </si>
+  <si>
+    <t>INFINIX SMART 10 128GB/4+4RAM - TWILIGHT GOLD (1389)</t>
+  </si>
+  <si>
+    <t>INFINIX SMART 6 64GB/2RAM - PRETO (891)</t>
+  </si>
+  <si>
+    <t>INFINIX HOT 60I 256GB/8+8RAM - TITANIUM SILVER (10000323)</t>
+  </si>
+  <si>
+    <t>IPHONE 14 PRO 256GB - GRAFITE (10000336)</t>
+  </si>
+  <si>
+    <t>ITEL A80 128GB/4RAM - AZUL (10000318)</t>
+  </si>
+  <si>
+    <t>REALME C71 128GB/4RAM - WHITE SWAN (10000320)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 256GB/8RAM - PRETO (10000313)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 256GB/8RAM - VERDE (10000314)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI 14C 256GB/8RAM - MIDNIGHT BLACK (10000335)</t>
+  </si>
+  <si>
+    <t>INFINIX SMART 8 PRO 256GB/8RAM - PRETO (1184)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK GO 1 128GB/4RAM - MAGIC SKIN GREEN (10000316)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI A5 4RAM/128GB - MIDNIGHT BLACK (10000173)</t>
+  </si>
+  <si>
+    <t>IPHONE 15 128GB BLACK (10000347)</t>
+  </si>
+  <si>
+    <t>POCO C65 256GB/8 RAM - PRETO (10000333)</t>
+  </si>
+  <si>
+    <t>REALME C73 NFC 128GB/4RAM - FOREST OWLP (1534)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 5G 256GB/8RAM - AZUL (1527)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 5G 256GB/8RAM - CINZA (1528)</t>
+  </si>
+  <si>
+    <t>REALME C73 NFC 128GB/4RAM - VIOLET PARROT (1533)</t>
+  </si>
+  <si>
+    <t>REALME C73 256GB - VIOLET PARROT (10000219)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD 2 128GB/4RAM GRAPHITE GRAY (10000212)</t>
+  </si>
+  <si>
+    <t>GALAXY A07 PRETO 128GB/4RAM (10000189)</t>
+  </si>
+  <si>
+    <t>POCO C75 256GB/8RAM - GOLD (10000340)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 5G 128GB/4RAM - PRETO (1525)</t>
+  </si>
+  <si>
+    <t>REALME C85 256GB/8RAM - KINGFISHER BLUE (10000321)</t>
+  </si>
+  <si>
+    <t>INFINIX SMART 9 128GB/8RAM - METALLIC BLACK (10000007)</t>
+  </si>
+  <si>
+    <t>IPHONE 11 128GB BLACK (365)</t>
+  </si>
+  <si>
+    <t>IPHONE 11 64GB - WHITE (196)</t>
+  </si>
+  <si>
+    <t>IPHONE 12 PRO 128GB - GOLD (1278)</t>
+  </si>
+  <si>
+    <t>IPHONE 12 PRO 128GB - GRAPHITE (1279)</t>
+  </si>
+  <si>
+    <t>IPHONE 13 PRO 128GB VITRINE- VERDE (691)</t>
+  </si>
+  <si>
+    <t>IPHONE 13 128GB - RED - VITRINE (454)</t>
+  </si>
+  <si>
+    <t>IPHONE 13 128GB-MIDNIGHT- VITRINE (911)</t>
+  </si>
+  <si>
+    <t>IPHONE 13 PRO 128GB - WHITE (VITRINE) (1280)</t>
+  </si>
+  <si>
+    <t>IPHONE 13 PRO 256GB - GRAFITE (VITRINE) (1281)</t>
+  </si>
+  <si>
+    <t>IPHONE 13 PRO MAX 128GB - BLUE (VITRINE) (842)</t>
+  </si>
+  <si>
+    <t>IPHONE 13 PRO MAX 128GB - GRAPHITE (VITRINE) (529)</t>
+  </si>
+  <si>
+    <t>IPHONE 13 PRO MAX 128GB - GREEN (VITRINE) (1282)</t>
+  </si>
+  <si>
+    <t>IPHONE 13 PRO MAX 256GB - BLUE (VITRINE) (310)</t>
+  </si>
+  <si>
+    <t>IPHONE 13 PRO MAX 256GB - GRAPHITE (VITRINE) (949)</t>
+  </si>
+  <si>
+    <t>IPHONE 13 STARLIGHT-128GB (288)</t>
+  </si>
+  <si>
+    <t>IPHONE 14 PRO MAX 128GB VITRINE - WHITE (10000014)</t>
+  </si>
+  <si>
+    <t>IPHONE 14 128GB PRETO - VITRINE (10000057)</t>
+  </si>
+  <si>
+    <t>IPHONE 14 256GB - MIDNIGHT (VITRINE) (877)</t>
+  </si>
+  <si>
+    <t>IPHONE 14 P128GB- STARLIGHT - VITRINE (10000077)</t>
+  </si>
+  <si>
+    <t>IPHONE 14 PRO MAX 128GB - WHITE VITRINE (10000075)</t>
+  </si>
+  <si>
+    <t>IPHONE 15 128GB - GREEN (762)</t>
+  </si>
+  <si>
+    <t>IPHONE 15 128GB BLACK - VITRINE (1258)</t>
+  </si>
+  <si>
+    <t>IPHONE 15 128GB BLACK (1175)</t>
+  </si>
+  <si>
+    <t>IPHONE 15 PRO 128GB - BLUE TITANIUM (VITRINE) (1284)</t>
+  </si>
+  <si>
+    <t>IPHONE 15 PRO 256GB - BLACK TITANIUM (VITRINE) (1283)</t>
+  </si>
+  <si>
+    <t>IPHONE 15 PRO MAX 256GB-NATURAL TITANIUM ( VITRINE) (1146)</t>
+  </si>
+  <si>
+    <t>IPHONE 15 PRO MAX 256GB-NATURAL TITANIUM (728)</t>
+  </si>
+  <si>
+    <t>IPHONE 16 128GB - BLACK (10000045)</t>
+  </si>
+  <si>
+    <t>IPHONE 16 128GB - TEAL (10000046)</t>
+  </si>
+  <si>
+    <t>IPHONE 16 128GB - TEAL (10000132)</t>
+  </si>
+  <si>
+    <t>IPHONE 16 128GB - PINK (1445)</t>
+  </si>
+  <si>
+    <t>IPHONE 16 128GB - TEAL (10000177)</t>
+  </si>
+  <si>
+    <t>IPHONE 16 PRO 512GB - NATURAL TITANIUM (10000190)</t>
+  </si>
+  <si>
+    <t>IPHONE 16 PRO 512GB - WHITE TITANIUM (10000044)</t>
+  </si>
+  <si>
+    <t>IPHONE 17 256GB - MIST BLUE (1447)</t>
+  </si>
+  <si>
+    <t>IPHONE 17 256GB - WHITE (10000247)</t>
+  </si>
+  <si>
+    <t>IPHONE 17 PRO MAX 256GB - SILVER (1518)</t>
+  </si>
+  <si>
+    <t>IPHONE 17 PRO MAX 256GB - DEEP BLUE (1449)</t>
+  </si>
+  <si>
+    <t>IPHONE 17 PRO MAX 256GB - COSMIC ORANGE (1448)</t>
+  </si>
+  <si>
+    <t>IPHONE XR 128GB WHITE-VITRINE (177)</t>
+  </si>
+  <si>
+    <t>IPHONE XR 64B BLACK - SEMI NOVO (765)</t>
+  </si>
+  <si>
+    <t>IPHONE XR 64B WHITE - SEMI NOVO (764)</t>
+  </si>
+  <si>
+    <t>ITEL A50 256GB \4RAM LIME GREEN (10000128)</t>
+  </si>
+  <si>
+    <t>ITEL A50 256GB \4RAM MISTY BLACK (10000129)</t>
+  </si>
+  <si>
+    <t>ITEL A80 128GB/4RAM - SANDSTONE BLACK (1494)</t>
+  </si>
+  <si>
+    <t>ITEL A80 128GB/4RAM - SANDSTONE PRETO (10000289)</t>
+  </si>
+  <si>
+    <t>ITEL A80 128GB/4RAM - WAVE BLUE (1495)</t>
+  </si>
+  <si>
+    <t>ITEL A90 128GB/4RAM - SPACE TITANIUM (1484)</t>
+  </si>
+  <si>
+    <t>ITEL A90 128GB/4RAM - AURORA BLUE (1487)</t>
+  </si>
+  <si>
+    <t>ITEL A90 128GB/4RAM - STARLIT BLACK (10000116)</t>
+  </si>
+  <si>
+    <t>ITEL A90 256 GB/4RAM - STARLIT BLACK (10000117)</t>
+  </si>
+  <si>
+    <t>KIT STARLINK MINI INTERNET VIA SATELITE (10000398)</t>
+  </si>
+  <si>
+    <t>MOTOROLA G05 128GB/4RAM - VIOLETA (10000167)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G04S 128GB/4RAM - CORAL (939)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G04S 128GB/4RAM - GRAFITE (985)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G05 128GB/4RAM - CINZA (240)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G06 128GB/4RAM - AZUL MARINHO (10000048)</t>
+  </si>
+  <si>
+    <t>MOTOROLA G06 LARANJA 128GB/4RAM (10000186)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G06 128GB/4RAM - AZUL MARINHO (1452)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G06 128GB/4RAM - LARANJA (10000049)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G06 128GB/4RAM - LARANJA (1453)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G06 256GB/4RAM - BEGE (10000102)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G06 256GB/4RAM - BEGE (10000188)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G06 268GB/4RAM - VERDE (10000189)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G14 128GB-GRAFITE (581)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G14 128GB-LILAC (558)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G15 256 GB/4RAM- VERDE (10000103)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G15 128GB/4RAM AZUL ESCURO (10000130)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G15 256GB/4RAM - GRAFITE (10000004)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G15 256GB/4RAM - GRAFITE (10000168)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G15 256GB/4RAM - VERDE (10000061)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G15 256GB/4RAM -GRAFITE (1260)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G23 128GB/4RAM- GRAFITE (363)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G24 128GB/4RAM - GRAFITE (832)</t>
+  </si>
+  <si>
+    <t>MOTOROLA MOTO G54 5G 256GB/8RAM - AZUL (987)</t>
+  </si>
+  <si>
+    <t>OPPO A40 256GB/4GB - CAFÉ (10000138)</t>
+  </si>
+  <si>
+    <t>OPPO A40 256GB/4GB - LILA (10000139)</t>
+  </si>
+  <si>
+    <t>OPPO A40 256GB/4RAM - LILA (10000076)</t>
+  </si>
+  <si>
+    <t>OPPO A60 256GB/8GB - BLANCO (10000140)</t>
+  </si>
+  <si>
+    <t>OPPO A60 256GB/8GB - NEGRO (10000141)</t>
+  </si>
+  <si>
+    <t>OPPO A60 256GB/8RAM - BLANCO (10000049)</t>
+  </si>
+  <si>
+    <t>OPPO A60 256GB/8RAM - NEGRO (10000050)</t>
+  </si>
+  <si>
+    <t>OUKITEL P1 256GB/8RAM - BLACK (1516)</t>
+  </si>
+  <si>
+    <t>OUKITEL P1 256GB/8RAM - GOLD (1517)</t>
+  </si>
+  <si>
+    <t>OUKITEL P1 PRO 512GB/8RAM - ORANGE (1488)</t>
+  </si>
+  <si>
+    <t>POCO C71 128GB/4RAM - AZUL (10000253)</t>
+  </si>
+  <si>
+    <t>POCO C71 4G 128GB/4RAM - AZUL (1353)</t>
+  </si>
+  <si>
+    <t>POCO C71 4G 128GB/4RAM - PRETO (1354)</t>
+  </si>
+  <si>
+    <t>POCO C71 64GB/3RAM - PRETO (10000055)</t>
+  </si>
+  <si>
+    <t>POCO C75 128GB/6+6RAM - DOURADO - ANATEL (1444)</t>
+  </si>
+  <si>
+    <t>POCO C75 128GB/6+6RAM - PRETO - ANATEL (1443)</t>
+  </si>
+  <si>
+    <t>POCO X7 PRO 5G 256GB/8RAM - BLACK (10000383)</t>
+  </si>
+  <si>
+    <t>POCO X7 PRO 256GB/8RAM - BLACK (10000058)</t>
+  </si>
+  <si>
+    <t>POCO X7 PRO 256GB/8RAM - YELLOW (10000059)</t>
+  </si>
+  <si>
+    <t>POCO X7 5G 256GB/8RAM GREEN (10000208)</t>
+  </si>
+  <si>
+    <t>POCO X7 PRO 5G 512GB/12RAM - BLACK (10000065)</t>
+  </si>
+  <si>
+    <t>POCO X7 PRO 5G 256GB/8RAM - GREEN (957)</t>
+  </si>
+  <si>
+    <t>POCO X7 PRO 5G 512GB/12RAM - AMARILLO/YELLOW (1335)</t>
+  </si>
+  <si>
+    <t>POCO X7 PRO 5G 512GB/12RAM - BLACK (10000225)</t>
+  </si>
+  <si>
+    <t>POCO X7 PRO 5G 512GB/12RAM - GREEN (10000215)</t>
+  </si>
+  <si>
+    <t>POCO X7 PRO 5G 512GB/12RAM - NEGRO (1398)</t>
+  </si>
+  <si>
+    <t>POCO X7 PRO IRON MAN 512GB/12RAM (1266)</t>
+  </si>
+  <si>
+    <t>POSITIVO TABLET TWIST TAB+ 64GB/2RAM (1112)</t>
+  </si>
+  <si>
+    <t>POSITIVO TABLET VISION TAB 7 MINIONS 64GB/3RAM (10000001)</t>
+  </si>
+  <si>
+    <t>POSITIVO TWIST TABLET TAB MINIONS+ 64GB/2RAM (1111)</t>
+  </si>
+  <si>
+    <t>POSITIVO TABLET VISION TAB 7 MINIONS 64GB/3RAM (10000068)</t>
+  </si>
+  <si>
+    <t>POSITIVO TABLET VISION TAB 7 MINIONS 64GB/3RAM (10000226)</t>
+  </si>
+  <si>
+    <t>POSITIVO TABLET VISION TAB 7 SPIDEY 64GB/3RAM (10000002)</t>
+  </si>
+  <si>
+    <t>POSITIVO TABLET VISION TAB 7 SPIDEY 64GB/3RAM (10000227)</t>
+  </si>
+  <si>
+    <t>POWER 3 256GB/16RAM- BLACK (10000084)</t>
+  </si>
+  <si>
+    <t>REALME (10000171)</t>
+  </si>
+  <si>
+    <t>REALME 12X (5G) 256GB/8RAM - FEATHER GREEN (1109)</t>
+  </si>
+  <si>
+    <t>REALME 14 5G 256GB/12RAM - STORM TITANIUM (1315)</t>
+  </si>
+  <si>
+    <t>REALME 14 5G 512GB/12RAM - WARRIOR PINK (1303)</t>
+  </si>
+  <si>
+    <t>REALME 14 PRO + 5G 512GB/12RAM - SUEDE GREY (10000213)</t>
+  </si>
+  <si>
+    <t>REALME C30 32GB/2GB- LAKE BLUE (446)</t>
+  </si>
+  <si>
+    <t>REALME C51 128GB/4RAM -MINT GREEN (713)</t>
+  </si>
+  <si>
+    <t>REALME C55 256GB 8GB - RAINY NIGHT (441)</t>
+  </si>
+  <si>
+    <t>REALME C61 256GB/6RAM - DARK GREEN (1256)</t>
+  </si>
+  <si>
+    <t>REALME C61 256GB/6RAM - SPARKLE GOLD (1255)</t>
+  </si>
+  <si>
+    <t>REALME C61 NFC 128GB/4RAM - DARK GREEN (10000077)</t>
+  </si>
+  <si>
+    <t>REALME C61 NFC 128GB/4RAM - DARK GREEN SEMINOVO (10000387)</t>
+  </si>
+  <si>
+    <t>REALME C61 NFC 128GB/4RAM - SPARKLE GOLD (10000011)</t>
+  </si>
+  <si>
+    <t>REALME C61 NFC 128GB/4RAM - SPARKLE GOLD (10000034)</t>
+  </si>
+  <si>
+    <t>REALME C61 NFC 256GB/8RAM - DARK GREEN (1119)</t>
+  </si>
+  <si>
+    <t>REALME C61 NFC 256GB/8RAM - SPARKLE GOLD (1126)</t>
+  </si>
+  <si>
+    <t>REALME C63 NFC 128GB/6RAM - JADE GREEN (1285)</t>
+  </si>
+  <si>
+    <t>REALME C63 NFC 128GB/6RAM - LEATHER BLUE (1486)</t>
+  </si>
+  <si>
+    <t>REALME C63 NFC 256GB/8RAM - LEATHER BLUE (10000290)</t>
+  </si>
+  <si>
+    <t>REALME C63 NFC 256GB/8RAM - JADE GREEN (1106)</t>
+  </si>
+  <si>
+    <t>REALME C63 NFC 256GB/8RAM - JADE VERDE (10000275)</t>
+  </si>
+  <si>
+    <t>REALME C63 NFC 128GB/6RAM - JADE VERDE (10000274)</t>
+  </si>
+  <si>
+    <t>REALME C63 NFC 256GB/8RAM - LEATHER BLUE (1105)</t>
+  </si>
+  <si>
+    <t>REALME C65 256GB/8 RAM - STARLIGHT BLACK (1253)</t>
+  </si>
+  <si>
+    <t>REALME C65 NFC 256GB/8RAM - STARLIGHT BLACK (10000082)</t>
+  </si>
+  <si>
+    <t>REALME C65 NFC 256GB/8RAM - STARLIGHT PURPLE (10000008)</t>
+  </si>
+  <si>
+    <t>REALME C67 256GB/8RAM- BLACK ROCK (830)</t>
+  </si>
+  <si>
+    <t>REALME C67 256GB/8RAM- SUNNY OASIS (813)</t>
+  </si>
+  <si>
+    <t>REALME C67 NFC 128GB/6RAM - BLACK ROCK (863)</t>
+  </si>
+  <si>
+    <t>REALME C71 NFC 128GB/4RAM - FOREST OWL (1432)</t>
+  </si>
+  <si>
+    <t>REALME C71 NFC 128GB/4RAM - WHITE SWAN (1433)</t>
+  </si>
+  <si>
+    <t>REALME C71 NFC 256GB/8RAM - WHITE SWAN (10000049)</t>
+  </si>
+  <si>
+    <t>REALME C71 NFC 256GB/8RAM - FOREST OWL (10000036)</t>
+  </si>
+  <si>
+    <t>REALME C71 NFC 256GB/8RAM - FOREST OWL (10000048)</t>
+  </si>
+  <si>
+    <t>REALME C71 NFC 128GB/4RAM FOREST OWL (10000214)</t>
+  </si>
+  <si>
+    <t>REALME C71 NFC 256GB/8RAM - WHITE SWAN (10000037)</t>
+  </si>
+  <si>
+    <t>REALME C73 NFC 256GB/8RAM - VIOLET PARROT (1499)</t>
+  </si>
+  <si>
+    <t>REALME C73 256GB/8RAM - VIOLET PARROT (1499)</t>
+  </si>
+  <si>
+    <t>REALME C75 NFC 256GB/8RAM - LIGHTNIG GOLD (10000061)</t>
+  </si>
+  <si>
+    <t>REALME C75 5G 256GB/8RAM - LIGHTNING GOLD (1438)</t>
+  </si>
+  <si>
+    <t>REALME C75 256GB/8RAM - LIGHTNING GOLD (10000168)</t>
+  </si>
+  <si>
+    <t>REALME C75 5G 256GB/8RAM - STORM BLACK (1437)</t>
+  </si>
+  <si>
+    <t>REALME C75 NFC 256GB/8RAM - LIGHTNING GOLD (10000027)</t>
+  </si>
+  <si>
+    <t>REALME C75 NFC 256GB/8RAM - LIGHTNING GOLD (10000176)</t>
+  </si>
+  <si>
+    <t>REALME C75 NFC 256GB/8RAM - RUBY RED (1429)</t>
+  </si>
+  <si>
+    <t>REALME C75 NFC 256GB/8RAM - STORM BLACK (1257)</t>
+  </si>
+  <si>
+    <t>REALME C75X NFC 256GB/8RAM - AZUL (10000293)</t>
+  </si>
+  <si>
+    <t>REALME C75X NFC 256GB/8RAM - CORAL PINK (1327)</t>
+  </si>
+  <si>
+    <t>REALME C75X 256GB/8RAM CORAL PINK (10000199)</t>
+  </si>
+  <si>
+    <t>REALME C75X NFC 256/8RAM - ROSA (10000292)</t>
+  </si>
+  <si>
+    <t>REALME C75X NFC 256GB/8RAM - OCEANIC BLUE (1328)</t>
+  </si>
+  <si>
+    <t>REALME C85 NFC 256GB/8RAM - KINGFISHER BLUE (1464)</t>
+  </si>
+  <si>
+    <t>REALME C85 256GB / 8RAM - PRETO (10000291)</t>
+  </si>
+  <si>
+    <t>REALME C85 256GB / 8RAM - SWAN PRETO (10000248)</t>
+  </si>
+  <si>
+    <t>REALME C85 NFC 256GB/8RAM - SWAN BLACK (1463)</t>
+  </si>
+  <si>
+    <t>REALME C85 PRO 256GB/8RAM - PARROT PURPLE (1462)</t>
+  </si>
+  <si>
+    <t>REALME C85 PRO 256GB/8RAM PARROT PURPLE (10000197)</t>
+  </si>
+  <si>
+    <t>REALME C85 PRO 256GB / 8RAM - PEACOCK GREEN (10000298)</t>
+  </si>
+  <si>
+    <t>REALME C85 PRO 256GB / 8RAM - PARROT PURPLE (10000299)</t>
+  </si>
+  <si>
+    <t>REALME C85 PRO 256GB/8RAM - PEACOCK GREEN (1482)</t>
+  </si>
+  <si>
+    <t>realme c85 (10000181)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 50 128GB/4RAM - MIDNIGHT BLACK (910)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 50 128GB/4RAM - SKY BLUE (909)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 50 64GB/3RAM - SKY BLUE (879)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 60 128GB/4GB - MARBLE BLACK (10000177)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 60 128GB/4RAM - MARBLE BLACK (1265)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 60 128GB/4RAM - VOYAGE BLUE (1264)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 60 256GB/4RAM - VOYAGE BLUE (10000080)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 60S 256GB/8RAM - SAFARI GREEN (1474)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 60X 128GB/4RAM - MARBLE BLACK (1347)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 60X 64GB/3RAM - MARBLE BLACK (1357)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 60X 64GB/3RAM - WILDERNESS GREEN (1385)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 60X 128GB/4RAM - WILDERNESS GREEN (1348)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 70 256GB/8RAM - BEACH GOLD (10000058)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 70 128GB/4RAM - GOLD (10000256)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 70 128GB/4RAM BEACH GOLD (10000207)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 70 128GB/4RAM - BEACH GOLD (1431)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 70 128GB/4RAM - PRETO (10000257)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 70 128GB/4RAM - OBSIDIAN BLACK (1430)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 70 256GB/8RAM - OBSIDIAN BLACK (10000059)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 70 256GB/8RAM - OBSIDIAN BLACK (10000249)</t>
+  </si>
+  <si>
+    <t>REALME NOTE 70S 128GB/4RAM - BEACH GOLD (1475)</t>
+  </si>
+  <si>
+    <t>REALME X50 5G 128GB/6GB- (25)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 256GB/8RAM - LIME VERDE (10000196)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 256GB/8GB- LIME GREEN (10000185)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 256GB/8RAM - MIDNIGHT BLACK (10000276)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 256GB/8RAM - LIME GREEN (10000217)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI NOTE 14 128GB/6RAM - MIST PURPLE (1247)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 256GB/8RAM - OCEAN BLUE (10000219)</t>
+  </si>
+  <si>
+    <t>REDMI 13C 128GB/4RAM ANATEL - AZUL (10000031)</t>
+  </si>
+  <si>
+    <t>REDMI 14C 128GB/4+4RAM - AZUL - ANATEL (1442)</t>
+  </si>
+  <si>
+    <t>REDMI 14C 128GB/4+4RAM - PRETO - ANATEL (10000241)</t>
+  </si>
+  <si>
+    <t>REDMI 14C 256GB/4+4RAM ANATEL - PRETO (10000029)</t>
+  </si>
+  <si>
+    <t>REDMI 14C 256GB/8RAM - MIDNIGHT BLACK (10000216)</t>
+  </si>
+  <si>
+    <t>REDMI 14C 256GB/8RAM - STARRY BLUE (10000047)</t>
+  </si>
+  <si>
+    <t>REDMI 14C 256GB/8RAM - STARRY BLUE (10000063)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 128 GB/4RAM - MINT GREEN (10000113)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 128GB/4RAM - MIDNIGHT BLACK (1461)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 128GB/6RAM - MIDNIGHT BLACK (10000295)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 128GB/4RAM - MOONLIGT BLUE (10000162)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 128GB/4RAM - MINT GREEN (10000161)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 256 GB/8RAM - MIDNIGHT BLUE (10000112)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 256GB/8RAM - MINT GREEN (10000255)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 5G 256GB/4+4RAM - PRETO - ANATEL (1425)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 5G 256GB/4+4RAM - ROXO - ANATEL (1423)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 5G 256GB/4+4RAM - VERDE - ANATEL (1424)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI 15 128GB/6RAM - MIDNIGHT BLACK (1508)</t>
+  </si>
+  <si>
+    <t>REDMI 15C G 256GB/4 AZUL LUNAR (10000111)</t>
+  </si>
+  <si>
+    <t>REDMI A3 128GB/4RAM - ANATEL - PRETO (10000134)</t>
+  </si>
+  <si>
+    <t>REDMI A3 128GB/4RAM - ANATEL - VERDE (10000133)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI A5 64GB/3RAM - SANDY GOLD (1304)</t>
+  </si>
+  <si>
+    <t>REDMI A5 128GB/4+4RAM - ANATEL - AZUL (10000242)</t>
+  </si>
+  <si>
+    <t>REDMI A5 128GB/4+4RAM - ANATEL - PRETO (10000239)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 13 256GB/8RAM ANATEL - PRETO (10000030)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 128GB/6GB - OCEAN BLUE (10000163)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 256GB/8+8RAM - AZUL - ANATEL (1441)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 256GB/8+8RAM - PRETO - ANATEL (10000240)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI NOTE 14 256GB/8RAM - VERDE LIMON (1334)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 256GB/8+8RAM - VERDE - ANATEL (10000176)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 256GB/8RAM - MIDNIGHT BLACK (10000155)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 256GB/8RAM - OCEAN BLUE (10000197)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 PRO 4G 256GB/8RAM - AZUL OCÉANO (1023)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 14 PRO 4G 256GB/8RAM - MIDNIGHT BLACK (1306)</t>
+  </si>
+  <si>
+    <t>REDMI 15C 256GB/8+8RAM - VERDE - ANATEL (1424)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI NOTE 15 256GB/8RAM - PURPLE (1510)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI NOTE 15 256GB/8RAM - FOREST GREEN (10000296)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 15 PRO 256GB 8GB/RAM - BLACK (10000288)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 15 PRO 256GB/8RAM - GACIER AZUL (10000310)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 15 256 GB/8RAM - GLACIER BLUE (10000114)</t>
+  </si>
+  <si>
+    <t>REDMI NOTE 15 256GB/8RAM - GACIER AZUL (10000251)</t>
+  </si>
+  <si>
+    <t>SAMSUNG A03 CORE 32GB/2GB - PRETO (535)</t>
+  </si>
+  <si>
+    <t>SAMSUNG A03 CORE 32GB/2RAM -COBRE (65)</t>
+  </si>
+  <si>
+    <t>SAMSUNG A04e 64GB-PRETO (332)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A05 128GB- PRATA (918)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A05S 128GB/6RAM - PRATA (1110)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A05S 128GB/6RAM - PRETO (1071)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A06 128GB/4GB - AZUL ESCURO (10000042)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A06 128GB/4RAM - AZUL ESCURO (1250)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A06 128GB/4RAM - BRANCO (10000005)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A06 128GB/4RAM - BRANCO (10000067)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A06 128GB/4RAM - BRANCO (10000119)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A06 128GB/4RAM - VERDE CLARO (10000025)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A07 128GB/4RAM - PRETO (10000053)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A07 128GB/4RAM - PRETO (1454)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A07 128GB/4RAM – VERDE (10000254)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A07 128GB/4RAM - VERDE (1435)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A07 128GB/4RAM - VIOLETA (1436)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A07 256GB/8RAM - PRETO (1455)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A14 128GB/4GB - VERDE LIMA (458)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A14 128GB/4GB - PRETO* (484)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A16 128GB/4RAM - PRETO (10000159)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A16 128GB/4RAM - PRETO (10000245)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A16 4G 128GB/4RAM - BLACK (10000078)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A16 4G 128GB/4RAM - CINZA (1249)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A16 4G 128GB/4RAM - PRETO (10000053)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A16 4G 128GB/4RAM - VERDE CLARO (1308)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A16 4G 128GB/4RAM - WHITE (10000079)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A16 128GB/4RAM - CINZA (1249)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 128GB/4RAM - CINZA (10000068)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 4G 128GB - PRETO (10000438)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 128GB/4RAM - PRETO (10000069)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 128GB/4RAM - PRETO (10000186)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 4G 128GB/4RAM - AZUL (1476)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 128GB/4RAM - CINZA (10000187)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 4G 128GB/4RAM - CINZA (1496)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 4G 256GB/8RAM - CINZA (1522)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 4G 256GB/8RAM - AZUL (1477)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A17 4GB 128GB/4RAM - PRETO 5G INTERNETE (10000125)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A26 5G 256GB/8RAM - BRANCO (1350)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A26 5G 256GB/8RAM - PRETO (1351)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A36 5G 256GB/8RAM - BRANCO (1497)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A36 5G 256GB/8RAM - VERDE (1478)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY A56 5G 256GB/8RAM - PRETO (1426)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY M14 5G 128GB-AZUL MARINHO (755)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY M14 5G 128GB-PRATA (756)</t>
+  </si>
+  <si>
+    <t>SAMSUNG GALAXY TAB A9 64GB/4RAM - GRAFITE (1375)</t>
+  </si>
+  <si>
+    <t>STARLINK - ANTENA (10000333)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD 2 128GB/4RAM - MINT GREEN (1520)</t>
+  </si>
+  <si>
+    <t>TABLET REALME PAD 2 128GB/6RAM - IMAGINATION GREY (1054)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD 2 256GB/8RAM - MINT GREEN (1481)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD SE 128GB/4GB - GRAPHITE GRAY (10000054)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD SE 128GB/4GB - GRAPHITE GRAY (10000111)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD SE 128GB/4GB - LAVENDER PURPLE (10000017)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD SE 128GB/4GB - MINT GREEN (1056)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD SE 128GB/4RAM - GRAPHITE GRAY (10000009)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD SE 256GB /8GB - GRAPHITE GRAY (10000121)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD SE 256GB/8RAM - GRAPHITE GRAY (1167)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD 2 128GB/4RAM - GRAPHITE GRAY (1519)</t>
+  </si>
+  <si>
+    <t>TABLET REDMI PAD SE 256GB/8RAM - MINT GREEN (1166)</t>
+  </si>
+  <si>
+    <t>TABLET SAMSUNG GALAXY TAB S6 64GB/4RAM -GRAFITE -LOJA (10000161)</t>
+  </si>
+  <si>
+    <t>TABLET SAMSUNG GALAXY TAB S6 LITE 64GB/4RAM - CINZA (10000021)</t>
+  </si>
+  <si>
+    <t>TABLET SAMSUNG GALAXY TAB S6 LITE 64GB/4RAM - ROSA (10000043)</t>
+  </si>
+  <si>
+    <t>TCL 40SE IN PLUS 256GB/12RAM - DARK GREY (1185)</t>
+  </si>
+  <si>
+    <t>TCL 605 128GB-4RAM - AZUL (10000164)</t>
+  </si>
+  <si>
+    <t>TECNO CAMON 30 5G 256GB/8RAM - BASALTIC DARK (1325)</t>
+  </si>
+  <si>
+    <t>TECNO CAMON 30 5G 256GB/8RAM - UYUNI SALT WHITE (1321)</t>
+  </si>
+  <si>
+    <t>TECNO POVA 7 4G 256GB/8RAM - MAGIC SILVER (1479)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK 30C 128GB/4RAM - MAGIC SKIN GREEN (1324)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK 30C 128GB/4RAM - ORBIT BLACK (1319)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK 30C 128GB/4RAM - ORBIT WHITE (1323)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK 30C 256GB/8RAM - MAGIC SKIN GREEN (1329)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK 30C 256GB/8RAM - ORBIT BLACK (10000279)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK 30C 256GB/8RAM - ORBIT BLACK (1330)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK 30C 256GB/8RAM - ORBIT WHITE (1331)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK GO 1 128GB / - SKIN GREEN (10000008)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK GO1 64GB/3RAM - GLITTERY WHITE (10000127)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK GO 1 128GB/4RAM - GLITTERY WHITE (1092)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK GO 1 128GB/4RAM - MAGIC SKIN GREEN (1365)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK GO 1 128GB/4RAM - STARTRAIL BLACK (1322)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK GO 1 64GB / 3GB - GLITTERY WHITE (10000024)</t>
+  </si>
+  <si>
+    <t>TECNO SPARK GO 1 64GB / 3GB - STARTRAIL BLACK (10000022)</t>
+  </si>
+  <si>
+    <t>teste (1358)</t>
+  </si>
+  <si>
+    <t>UMIDIGI NOTE 90A 64GB/4RAM GALAXY WHITY BRANCO (10000195)</t>
+  </si>
+  <si>
+    <t>POCO C65 256GB/8RAM- BLACK (10000027)</t>
+  </si>
+  <si>
+    <t>XIAOMI POCO C71 128GB/4RAM - BLUE (10000057)</t>
+  </si>
+  <si>
+    <t>POCO C71 128GB/4RAM - PRETO (10000252)</t>
+  </si>
+  <si>
+    <t>XIAOMI POCO C71 128GB/4RAM - GOLD (10000056)</t>
+  </si>
+  <si>
+    <t>POCO C71 4G 64GB/3RAM - AZUL (10000004)</t>
+  </si>
+  <si>
+    <t>POCO C71 4G 64GB/4RAM - DOURADO (10000005)</t>
+  </si>
+  <si>
+    <t>XIAOMI POCO C85 256GB/8RAM - MORADO (10000065)</t>
+  </si>
+  <si>
+    <t>XIAOMI POCO C85 256GB/8RAM - SWAN BLACK (10000064)</t>
+  </si>
+  <si>
+    <t>XIAOMI POCO X5 5G 256GB/8RAM- GREEN (344)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI NOTE 14 128GB/6RAM - LIME GREEN (1247)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI 13C 256GB/8RAM - CLOVER GREEN (676)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI 14C 128GB/4RAM - MIDNIGHT BLACK (10000008)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI 14C 128GB/4RAM - MIDNIGHT BLACK (10000234)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI 14C 128GB/4RAM - STARRY AZUL (10000258)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI A3 128GB/4RAM - FOREST GREEN (1309)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI A3 64GB/3RAM - NEGRO OCASO (903)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI A5 128GB/4+4RAM - MIDNIGHT BLACK (1287)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI A5 128GB/4+4RAM - OCEAN BLUE (1288)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI A5 128GB/4+4RAM - SANDY GOLD (1314)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI A5 64GB/3RAM - AZUL OCÉANO (1312)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI A5 64GB/3RAM - OCEAN BLUE (1298)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI NOTE 12 128GB/4RAM- ONYX GRAY (346)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI NOTE 12S 256GB 8GB RAM - ICE BLUE (440)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI NOTE 14 128GB/6RAM - MIDNIGHT BLACK (1248)</t>
+  </si>
+  <si>
+    <t>XIAOMI REDMI NOTE 14 128GB/6RAM - OCEAN BLUE (1246)</t>
+  </si>
+  <si>
+    <t>ZTE R236 - BRANCO/AZUL (816)</t>
+  </si>
+  <si>
+    <t>ZTE R236 - PRETO/VERMELHO (817)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
+  </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1894,7 +3146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1919,14 +3171,19 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="12" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1953,6 +3210,17 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{31E742E3-7121-4E61-9E37-043D773500FA}" name="Tabela1" displayName="Tabela1" ref="A1:B416" totalsRowShown="0">
+  <autoFilter ref="A1:B416" xr:uid="{31E742E3-7121-4E61-9E37-043D773500FA}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{F47EA37D-5B03-4F5C-AD30-FECFDECFDE35}" name="PRODUTO"/>
+    <tableColumn id="2" xr3:uid="{35007468-9DCA-4B08-82F5-4E43B72A3EDD}" name="PREÇO" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F8A0E3CE-1BCF-445A-90B7-CC16ED38CC14}" name="Tabela19" displayName="Tabela19" ref="A1:B7" totalsRowShown="0">
   <autoFilter ref="A1:B7" xr:uid="{F8A0E3CE-1BCF-445A-90B7-CC16ED38CC14}"/>
   <tableColumns count="2">
@@ -2625,6 +3893,3351 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4960596-8DB1-47AE-A3EA-DC840E831A8B}">
+  <dimension ref="A1:B416"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="65.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>563</v>
+      </c>
+      <c r="B1" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B2" s="27">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>566</v>
+      </c>
+      <c r="B3" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>567</v>
+      </c>
+      <c r="B4" s="27">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>568</v>
+      </c>
+      <c r="B5" s="27">
+        <v>179.99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>569</v>
+      </c>
+      <c r="B6" s="27">
+        <v>215.71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>570</v>
+      </c>
+      <c r="B7" s="27">
+        <v>149.99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>571</v>
+      </c>
+      <c r="B8" s="27">
+        <v>149.99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>572</v>
+      </c>
+      <c r="B9" s="27">
+        <v>379.99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>573</v>
+      </c>
+      <c r="B10" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>574</v>
+      </c>
+      <c r="B11" s="27">
+        <v>3599.99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>575</v>
+      </c>
+      <c r="B12" s="27">
+        <v>274.99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>576</v>
+      </c>
+      <c r="B13" s="27">
+        <v>3899.99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>577</v>
+      </c>
+      <c r="B14" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>578</v>
+      </c>
+      <c r="B15" s="27">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>579</v>
+      </c>
+      <c r="B16" s="27">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>580</v>
+      </c>
+      <c r="B17" s="27">
+        <v>897.16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>581</v>
+      </c>
+      <c r="B18" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>582</v>
+      </c>
+      <c r="B19" s="27">
+        <v>1695.31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>583</v>
+      </c>
+      <c r="B20" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>584</v>
+      </c>
+      <c r="B21" s="27">
+        <v>2399.9899999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>585</v>
+      </c>
+      <c r="B22" s="27">
+        <v>3599.99</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>586</v>
+      </c>
+      <c r="B23" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>587</v>
+      </c>
+      <c r="B24" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>588</v>
+      </c>
+      <c r="B25" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>589</v>
+      </c>
+      <c r="B26" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>590</v>
+      </c>
+      <c r="B27" s="27">
+        <v>1699.99</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>591</v>
+      </c>
+      <c r="B28" s="27">
+        <v>3199.99</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>592</v>
+      </c>
+      <c r="B29" s="27">
+        <v>1919.99</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>593</v>
+      </c>
+      <c r="B30" s="27">
+        <v>1919.99</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>594</v>
+      </c>
+      <c r="B31" s="27">
+        <v>1919.99</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>595</v>
+      </c>
+      <c r="B32" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>596</v>
+      </c>
+      <c r="B33" s="27">
+        <v>1687.49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>597</v>
+      </c>
+      <c r="B34" s="27">
+        <v>1687.49</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>598</v>
+      </c>
+      <c r="B35" s="27">
+        <v>2106.2399999999998</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>599</v>
+      </c>
+      <c r="B36" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>565</v>
+      </c>
+      <c r="B37" s="27">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>600</v>
+      </c>
+      <c r="B38" s="27">
+        <v>1124.99</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>601</v>
+      </c>
+      <c r="B39" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>602</v>
+      </c>
+      <c r="B40" s="27">
+        <v>1018.75</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>603</v>
+      </c>
+      <c r="B41" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>604</v>
+      </c>
+      <c r="B42" s="27">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>605</v>
+      </c>
+      <c r="B43" s="27">
+        <v>799.99</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>606</v>
+      </c>
+      <c r="B44" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>607</v>
+      </c>
+      <c r="B45" s="27">
+        <v>3550</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>608</v>
+      </c>
+      <c r="B46" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>609</v>
+      </c>
+      <c r="B47" s="27">
+        <v>1599.99</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>610</v>
+      </c>
+      <c r="B48" s="27">
+        <v>1899.99</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>611</v>
+      </c>
+      <c r="B49" s="27">
+        <v>1899.99</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>612</v>
+      </c>
+      <c r="B50" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>613</v>
+      </c>
+      <c r="B51" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>614</v>
+      </c>
+      <c r="B52" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>615</v>
+      </c>
+      <c r="B53" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>616</v>
+      </c>
+      <c r="B54" s="27">
+        <v>6999.99</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>617</v>
+      </c>
+      <c r="B55" s="27">
+        <v>1599.99</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>618</v>
+      </c>
+      <c r="B56" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>619</v>
+      </c>
+      <c r="B57" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>620</v>
+      </c>
+      <c r="B58" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>621</v>
+      </c>
+      <c r="B59" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>622</v>
+      </c>
+      <c r="B60" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>623</v>
+      </c>
+      <c r="B61" s="27">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>624</v>
+      </c>
+      <c r="B62" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>625</v>
+      </c>
+      <c r="B63" s="27">
+        <v>2699.99</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>626</v>
+      </c>
+      <c r="B64" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>627</v>
+      </c>
+      <c r="B65" s="27">
+        <v>2399.9899999999998</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>628</v>
+      </c>
+      <c r="B66" s="27">
+        <v>899.99</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>629</v>
+      </c>
+      <c r="B67" s="27">
+        <v>4000.17</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>630</v>
+      </c>
+      <c r="B68" s="27">
+        <v>3707.88</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>631</v>
+      </c>
+      <c r="B69" s="27">
+        <v>3750</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>632</v>
+      </c>
+      <c r="B70" s="27">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>633</v>
+      </c>
+      <c r="B71" s="27">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>634</v>
+      </c>
+      <c r="B72" s="27">
+        <v>4299.99</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>635</v>
+      </c>
+      <c r="B73" s="27">
+        <v>4299.99</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>636</v>
+      </c>
+      <c r="B74" s="27">
+        <v>3750</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>637</v>
+      </c>
+      <c r="B75" s="27">
+        <v>3950</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>638</v>
+      </c>
+      <c r="B76" s="27">
+        <v>4124.91</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>639</v>
+      </c>
+      <c r="B77" s="27">
+        <v>4171</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>640</v>
+      </c>
+      <c r="B78" s="27">
+        <v>4300</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>641</v>
+      </c>
+      <c r="B79" s="27">
+        <v>4363.51</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>642</v>
+      </c>
+      <c r="B80" s="27">
+        <v>4049.04</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>643</v>
+      </c>
+      <c r="B81" s="27">
+        <v>3459.86</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>644</v>
+      </c>
+      <c r="B82" s="27">
+        <v>7999.99</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>645</v>
+      </c>
+      <c r="B83" s="27">
+        <v>3299.99</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>646</v>
+      </c>
+      <c r="B84" s="27">
+        <v>3550</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>647</v>
+      </c>
+      <c r="B85" s="27">
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>648</v>
+      </c>
+      <c r="B86" s="27">
+        <v>6999.99</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>649</v>
+      </c>
+      <c r="B87" s="27">
+        <v>6999.99</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>650</v>
+      </c>
+      <c r="B88" s="27">
+        <v>6299.99</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>651</v>
+      </c>
+      <c r="B89" s="27">
+        <v>6999.99</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>652</v>
+      </c>
+      <c r="B90" s="27">
+        <v>5650</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>653</v>
+      </c>
+      <c r="B91" s="27">
+        <v>5950</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>654</v>
+      </c>
+      <c r="B92" s="27">
+        <v>6300</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>655</v>
+      </c>
+      <c r="B93" s="27">
+        <v>6600</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>656</v>
+      </c>
+      <c r="B94" s="27">
+        <v>7799.99</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>657</v>
+      </c>
+      <c r="B95" s="27">
+        <v>7799.99</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>658</v>
+      </c>
+      <c r="B96" s="27">
+        <v>6999.99</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>659</v>
+      </c>
+      <c r="B97" s="27">
+        <v>7799.99</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>660</v>
+      </c>
+      <c r="B98" s="27">
+        <v>4700</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>661</v>
+      </c>
+      <c r="B99" s="27">
+        <v>10999.99</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>662</v>
+      </c>
+      <c r="B100" s="27">
+        <v>10999.99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>663</v>
+      </c>
+      <c r="B101" s="27">
+        <v>8666.66</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>664</v>
+      </c>
+      <c r="B102" s="27">
+        <v>6999.99</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>665</v>
+      </c>
+      <c r="B103" s="27">
+        <v>10600</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>666</v>
+      </c>
+      <c r="B104" s="27">
+        <v>10600</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>667</v>
+      </c>
+      <c r="B105" s="27">
+        <v>10600</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>668</v>
+      </c>
+      <c r="B106" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>669</v>
+      </c>
+      <c r="B107" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>670</v>
+      </c>
+      <c r="B108" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>671</v>
+      </c>
+      <c r="B109" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
+        <v>672</v>
+      </c>
+      <c r="B110" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>673</v>
+      </c>
+      <c r="B111" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>674</v>
+      </c>
+      <c r="B112" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>675</v>
+      </c>
+      <c r="B113" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>676</v>
+      </c>
+      <c r="B114" s="27">
+        <v>1001.17</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>677</v>
+      </c>
+      <c r="B115" s="27">
+        <v>1001.17</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>678</v>
+      </c>
+      <c r="B116" s="27">
+        <v>1399.99</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
+        <v>679</v>
+      </c>
+      <c r="B117" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
+        <v>680</v>
+      </c>
+      <c r="B118" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>681</v>
+      </c>
+      <c r="B119" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
+        <v>682</v>
+      </c>
+      <c r="B120" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
+        <v>683</v>
+      </c>
+      <c r="B121" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>684</v>
+      </c>
+      <c r="B122" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>685</v>
+      </c>
+      <c r="B123" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
+        <v>686</v>
+      </c>
+      <c r="B124" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
+        <v>687</v>
+      </c>
+      <c r="B125" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>688</v>
+      </c>
+      <c r="B126" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
+        <v>689</v>
+      </c>
+      <c r="B127" s="27">
+        <v>1013.89</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
+        <v>690</v>
+      </c>
+      <c r="B128" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A129" t="s">
+        <v>691</v>
+      </c>
+      <c r="B129" s="27">
+        <v>1399.99</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A130" t="s">
+        <v>692</v>
+      </c>
+      <c r="B130" s="27">
+        <v>1399.99</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A131" t="s">
+        <v>693</v>
+      </c>
+      <c r="B131" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A132" t="s">
+        <v>694</v>
+      </c>
+      <c r="B132" s="27">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>695</v>
+      </c>
+      <c r="B133" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>696</v>
+      </c>
+      <c r="B134" s="27">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>697</v>
+      </c>
+      <c r="B135" s="27">
+        <v>1699.99</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
+        <v>698</v>
+      </c>
+      <c r="B136" s="27">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>699</v>
+      </c>
+      <c r="B137" s="27">
+        <v>1699.99</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>700</v>
+      </c>
+      <c r="B138" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>701</v>
+      </c>
+      <c r="B139" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
+        <v>702</v>
+      </c>
+      <c r="B140" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>703</v>
+      </c>
+      <c r="B141" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>704</v>
+      </c>
+      <c r="B142" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>705</v>
+      </c>
+      <c r="B143" s="27">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>706</v>
+      </c>
+      <c r="B144" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>707</v>
+      </c>
+      <c r="B145" s="27">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>708</v>
+      </c>
+      <c r="B146" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>709</v>
+      </c>
+      <c r="B147" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A148" t="s">
+        <v>710</v>
+      </c>
+      <c r="B148" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A149" t="s">
+        <v>711</v>
+      </c>
+      <c r="B149" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
+        <v>712</v>
+      </c>
+      <c r="B150" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
+        <v>713</v>
+      </c>
+      <c r="B151" s="27">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
+        <v>714</v>
+      </c>
+      <c r="B152" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
+        <v>715</v>
+      </c>
+      <c r="B153" s="27">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A154" t="s">
+        <v>716</v>
+      </c>
+      <c r="B154" s="27">
+        <v>1299.5</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>717</v>
+      </c>
+      <c r="B155" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>718</v>
+      </c>
+      <c r="B156" s="27">
+        <v>2699.99</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>719</v>
+      </c>
+      <c r="B157" s="27">
+        <v>2699.99</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>720</v>
+      </c>
+      <c r="B158" s="27">
+        <v>2999.99</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
+        <v>721</v>
+      </c>
+      <c r="B159" s="27">
+        <v>3499</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
+        <v>722</v>
+      </c>
+      <c r="B160" s="27">
+        <v>3499</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
+        <v>723</v>
+      </c>
+      <c r="B161" s="27">
+        <v>2999.99</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A162" t="s">
+        <v>724</v>
+      </c>
+      <c r="B162" s="27">
+        <v>4499.99</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A163" t="s">
+        <v>725</v>
+      </c>
+      <c r="B163" s="27">
+        <v>3266.66</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A164" t="s">
+        <v>726</v>
+      </c>
+      <c r="B164" s="27">
+        <v>3400</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A165" t="s">
+        <v>727</v>
+      </c>
+      <c r="B165" s="27">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A166" t="s">
+        <v>728</v>
+      </c>
+      <c r="B166" s="27">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A167" t="s">
+        <v>729</v>
+      </c>
+      <c r="B167" s="27">
+        <v>3999.99</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A168" t="s">
+        <v>730</v>
+      </c>
+      <c r="B168" s="27">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A169" t="s">
+        <v>731</v>
+      </c>
+      <c r="B169" s="27">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A170" t="s">
+        <v>732</v>
+      </c>
+      <c r="B170" s="27">
+        <v>899.99</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A171" t="s">
+        <v>733</v>
+      </c>
+      <c r="B171" s="27">
+        <v>699.99</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A172" t="s">
+        <v>734</v>
+      </c>
+      <c r="B172" s="27">
+        <v>699.99</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>735</v>
+      </c>
+      <c r="B173" s="27">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A174" t="s">
+        <v>736</v>
+      </c>
+      <c r="B174" s="27">
+        <v>899.99</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A175" t="s">
+        <v>737</v>
+      </c>
+      <c r="B175" s="27">
+        <v>699.99</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A176" t="s">
+        <v>738</v>
+      </c>
+      <c r="B176" s="27">
+        <v>2999.99</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A177" t="s">
+        <v>739</v>
+      </c>
+      <c r="B177" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A178" t="s">
+        <v>740</v>
+      </c>
+      <c r="B178" s="27">
+        <v>2599.9899999999998</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A179" t="s">
+        <v>741</v>
+      </c>
+      <c r="B179" s="27">
+        <v>2175</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A180" t="s">
+        <v>742</v>
+      </c>
+      <c r="B180" s="27">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A181" t="s">
+        <v>743</v>
+      </c>
+      <c r="B181" s="27">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A182" t="s">
+        <v>744</v>
+      </c>
+      <c r="B182" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A183" t="s">
+        <v>745</v>
+      </c>
+      <c r="B183" s="27">
+        <v>1599.99</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A184" t="s">
+        <v>746</v>
+      </c>
+      <c r="B184" s="27">
+        <v>2599.9899999999998</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A185" t="s">
+        <v>747</v>
+      </c>
+      <c r="B185" s="27">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A186" t="s">
+        <v>748</v>
+      </c>
+      <c r="B186" s="27">
+        <v>1766.66</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A187" t="s">
+        <v>749</v>
+      </c>
+      <c r="B187" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A188" t="s">
+        <v>750</v>
+      </c>
+      <c r="B188" s="27">
+        <v>899.99</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A189" t="s">
+        <v>751</v>
+      </c>
+      <c r="B189" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A190" t="s">
+        <v>752</v>
+      </c>
+      <c r="B190" s="27">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A191" t="s">
+        <v>753</v>
+      </c>
+      <c r="B191" s="27">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>754</v>
+      </c>
+      <c r="B192" s="27">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A193" t="s">
+        <v>755</v>
+      </c>
+      <c r="B193" s="27">
+        <v>1691.57</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A194" t="s">
+        <v>756</v>
+      </c>
+      <c r="B194" s="27">
+        <v>1712.49</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A195" t="s">
+        <v>757</v>
+      </c>
+      <c r="B195" s="27">
+        <v>1899.99</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A196" t="s">
+        <v>758</v>
+      </c>
+      <c r="B196" s="27">
+        <v>1899.99</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A197" t="s">
+        <v>759</v>
+      </c>
+      <c r="B197" s="27">
+        <v>1699.99</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A198" t="s">
+        <v>760</v>
+      </c>
+      <c r="B198" s="27">
+        <v>1699.99</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A199" t="s">
+        <v>761</v>
+      </c>
+      <c r="B199" s="27">
+        <v>1899.99</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
+        <v>762</v>
+      </c>
+      <c r="B200" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
+        <v>763</v>
+      </c>
+      <c r="B201" s="27">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A202" t="s">
+        <v>764</v>
+      </c>
+      <c r="B202" s="27">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A203" t="s">
+        <v>765</v>
+      </c>
+      <c r="B203" s="27">
+        <v>1571.43</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A204" t="s">
+        <v>766</v>
+      </c>
+      <c r="B204" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A205" t="s">
+        <v>767</v>
+      </c>
+      <c r="B205" s="27">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A206" t="s">
+        <v>768</v>
+      </c>
+      <c r="B206" s="27">
+        <v>1749.5</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A207" t="s">
+        <v>769</v>
+      </c>
+      <c r="B207" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A208" t="s">
+        <v>770</v>
+      </c>
+      <c r="B208" s="27">
+        <v>1899</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A209" t="s">
+        <v>771</v>
+      </c>
+      <c r="B209" s="27">
+        <v>1899</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A210" t="s">
+        <v>772</v>
+      </c>
+      <c r="B210" s="27">
+        <v>1749.5</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A211" t="s">
+        <v>773</v>
+      </c>
+      <c r="B211" s="27">
+        <v>1749.5</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A212" t="s">
+        <v>774</v>
+      </c>
+      <c r="B212" s="27">
+        <v>1899</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A213" t="s">
+        <v>775</v>
+      </c>
+      <c r="B213" s="27">
+        <v>1947.36</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A214" t="s">
+        <v>776</v>
+      </c>
+      <c r="B214" s="27">
+        <v>1947.36</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A215" t="s">
+        <v>777</v>
+      </c>
+      <c r="B215" s="27">
+        <v>2699.99</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A216" t="s">
+        <v>778</v>
+      </c>
+      <c r="B216" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A217" t="s">
+        <v>779</v>
+      </c>
+      <c r="B217" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A218" t="s">
+        <v>780</v>
+      </c>
+      <c r="B218" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A219" t="s">
+        <v>781</v>
+      </c>
+      <c r="B219" s="27">
+        <v>2499</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A220" t="s">
+        <v>782</v>
+      </c>
+      <c r="B220" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A221" t="s">
+        <v>783</v>
+      </c>
+      <c r="B221" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A222" t="s">
+        <v>784</v>
+      </c>
+      <c r="B222" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A223" t="s">
+        <v>785</v>
+      </c>
+      <c r="B223" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A224" t="s">
+        <v>786</v>
+      </c>
+      <c r="B224" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A225" t="s">
+        <v>787</v>
+      </c>
+      <c r="B225" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A226" t="s">
+        <v>788</v>
+      </c>
+      <c r="B226" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A227" t="s">
+        <v>789</v>
+      </c>
+      <c r="B227" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A228" t="s">
+        <v>790</v>
+      </c>
+      <c r="B228" s="27">
+        <v>2399.9899999999998</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A229" t="s">
+        <v>791</v>
+      </c>
+      <c r="B229" s="27">
+        <v>2399.9899999999998</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A230" t="s">
+        <v>792</v>
+      </c>
+      <c r="B230" s="27">
+        <v>2399.9899999999998</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A231" t="s">
+        <v>793</v>
+      </c>
+      <c r="B231" s="27">
+        <v>2399.9899999999998</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A232" t="s">
+        <v>794</v>
+      </c>
+      <c r="B232" s="27">
+        <v>2599.9899999999998</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A233" t="s">
+        <v>795</v>
+      </c>
+      <c r="B233" s="27">
+        <v>2599.9899999999998</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A234" t="s">
+        <v>796</v>
+      </c>
+      <c r="B234" s="27">
+        <v>2599.9899999999998</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A235" t="s">
+        <v>797</v>
+      </c>
+      <c r="B235" s="27">
+        <v>2599.9899999999998</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A236" t="s">
+        <v>798</v>
+      </c>
+      <c r="B236" s="27">
+        <v>2599.9899999999998</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A237" t="s">
+        <v>799</v>
+      </c>
+      <c r="B237" s="27">
+        <v>2469.9899999999998</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A238" t="s">
+        <v>800</v>
+      </c>
+      <c r="B238" s="27">
+        <v>1699.99</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A239" t="s">
+        <v>801</v>
+      </c>
+      <c r="B239" s="27">
+        <v>1699.99</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A240" t="s">
+        <v>802</v>
+      </c>
+      <c r="B240" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A241" t="s">
+        <v>803</v>
+      </c>
+      <c r="B241" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A242" t="s">
+        <v>804</v>
+      </c>
+      <c r="B242" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A243" t="s">
+        <v>805</v>
+      </c>
+      <c r="B243" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A244" t="s">
+        <v>806</v>
+      </c>
+      <c r="B244" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A245" t="s">
+        <v>807</v>
+      </c>
+      <c r="B245" s="27">
+        <v>1371.99</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A246" t="s">
+        <v>808</v>
+      </c>
+      <c r="B246" s="27">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A247" t="s">
+        <v>809</v>
+      </c>
+      <c r="B247" s="27">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A248" t="s">
+        <v>810</v>
+      </c>
+      <c r="B248" s="27">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A249" t="s">
+        <v>811</v>
+      </c>
+      <c r="B249" s="27">
+        <v>1033.8699999999999</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A250" t="s">
+        <v>812</v>
+      </c>
+      <c r="B250" s="27">
+        <v>1599.99</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A251" t="s">
+        <v>813</v>
+      </c>
+      <c r="B251" s="27">
+        <v>1399.99</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A252" t="s">
+        <v>814</v>
+      </c>
+      <c r="B252" s="27">
+        <v>1474.99</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A253" t="s">
+        <v>815</v>
+      </c>
+      <c r="B253" s="27">
+        <v>1474.99</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A254" t="s">
+        <v>816</v>
+      </c>
+      <c r="B254" s="27">
+        <v>1399.99</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A255" t="s">
+        <v>817</v>
+      </c>
+      <c r="B255" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A256" t="s">
+        <v>818</v>
+      </c>
+      <c r="B256" s="27">
+        <v>1599.99</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A257" t="s">
+        <v>819</v>
+      </c>
+      <c r="B257" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A258" t="s">
+        <v>820</v>
+      </c>
+      <c r="B258" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A259" t="s">
+        <v>821</v>
+      </c>
+      <c r="B259" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A260" t="s">
+        <v>822</v>
+      </c>
+      <c r="B260" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A261" t="s">
+        <v>823</v>
+      </c>
+      <c r="B261" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A262" t="s">
+        <v>824</v>
+      </c>
+      <c r="B262" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A263" t="s">
+        <v>825</v>
+      </c>
+      <c r="B263" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A264" t="s">
+        <v>826</v>
+      </c>
+      <c r="B264" s="27">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A265" t="s">
+        <v>827</v>
+      </c>
+      <c r="B265" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A266" t="s">
+        <v>828</v>
+      </c>
+      <c r="B266" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A267" t="s">
+        <v>829</v>
+      </c>
+      <c r="B267" s="27">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A268" t="s">
+        <v>830</v>
+      </c>
+      <c r="B268" s="27">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A269" t="s">
+        <v>831</v>
+      </c>
+      <c r="B269" s="27">
+        <v>1587.12</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A270" t="s">
+        <v>832</v>
+      </c>
+      <c r="B270" s="27">
+        <v>1699.99</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A271" t="s">
+        <v>833</v>
+      </c>
+      <c r="B271" s="27">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A272" t="s">
+        <v>834</v>
+      </c>
+      <c r="B272" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A273" t="s">
+        <v>835</v>
+      </c>
+      <c r="B273" s="27">
+        <v>1599</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A274" t="s">
+        <v>836</v>
+      </c>
+      <c r="B274" s="27">
+        <v>1599</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A275" t="s">
+        <v>837</v>
+      </c>
+      <c r="B275" s="27">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A276" t="s">
+        <v>838</v>
+      </c>
+      <c r="B276" s="27">
+        <v>1599</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A277" t="s">
+        <v>839</v>
+      </c>
+      <c r="B277" s="27">
+        <v>1599</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A278" t="s">
+        <v>840</v>
+      </c>
+      <c r="B278" s="27">
+        <v>1899</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A279" t="s">
+        <v>841</v>
+      </c>
+      <c r="B279" s="27">
+        <v>1599.99</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A280" t="s">
+        <v>842</v>
+      </c>
+      <c r="B280" s="27">
+        <v>2299</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A281" t="s">
+        <v>843</v>
+      </c>
+      <c r="B281" s="27">
+        <v>2533.33</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A282" t="s">
+        <v>844</v>
+      </c>
+      <c r="B282" s="27">
+        <v>2533.33</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A283" t="s">
+        <v>845</v>
+      </c>
+      <c r="B283" s="27">
+        <v>2299</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A284" t="s">
+        <v>846</v>
+      </c>
+      <c r="B284" s="27">
+        <v>1799</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A285" t="s">
+        <v>847</v>
+      </c>
+      <c r="B285" s="27">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A286" t="s">
+        <v>848</v>
+      </c>
+      <c r="B286" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A287" t="s">
+        <v>849</v>
+      </c>
+      <c r="B287" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A288" t="s">
+        <v>850</v>
+      </c>
+      <c r="B288" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A289" t="s">
+        <v>851</v>
+      </c>
+      <c r="B289" s="27">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A290" t="s">
+        <v>852</v>
+      </c>
+      <c r="B290" s="27">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A291" t="s">
+        <v>853</v>
+      </c>
+      <c r="B291" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A292" t="s">
+        <v>854</v>
+      </c>
+      <c r="B292" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A293" t="s">
+        <v>855</v>
+      </c>
+      <c r="B293" s="27">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A294" t="s">
+        <v>856</v>
+      </c>
+      <c r="B294" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A295" t="s">
+        <v>857</v>
+      </c>
+      <c r="B295" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A296" t="s">
+        <v>858</v>
+      </c>
+      <c r="B296" s="27">
+        <v>2299.9899999999998</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A297" t="s">
+        <v>859</v>
+      </c>
+      <c r="B297" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A298" t="s">
+        <v>860</v>
+      </c>
+      <c r="B298" s="27">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A299" t="s">
+        <v>861</v>
+      </c>
+      <c r="B299" s="27">
+        <v>2985.71</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A300" t="s">
+        <v>862</v>
+      </c>
+      <c r="B300" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A301" t="s">
+        <v>863</v>
+      </c>
+      <c r="B301" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A302" t="s">
+        <v>864</v>
+      </c>
+      <c r="B302" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A303" t="s">
+        <v>865</v>
+      </c>
+      <c r="B303" s="27">
+        <v>2999.99</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A304" t="s">
+        <v>866</v>
+      </c>
+      <c r="B304" s="27">
+        <v>2999.99</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A305" t="s">
+        <v>867</v>
+      </c>
+      <c r="B305" s="27">
+        <v>2799</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A306" t="s">
+        <v>868</v>
+      </c>
+      <c r="B306" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A307" t="s">
+        <v>869</v>
+      </c>
+      <c r="B307" s="27">
+        <v>599.99</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A308" t="s">
+        <v>870</v>
+      </c>
+      <c r="B308" s="27">
+        <v>599.99</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A309" t="s">
+        <v>871</v>
+      </c>
+      <c r="B309" s="27">
+        <v>899.99</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A310" t="s">
+        <v>872</v>
+      </c>
+      <c r="B310" s="27">
+        <v>1099.99</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A311" t="s">
+        <v>873</v>
+      </c>
+      <c r="B311" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A312" t="s">
+        <v>874</v>
+      </c>
+      <c r="B312" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A313" t="s">
+        <v>875</v>
+      </c>
+      <c r="B313" s="27">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A314" t="s">
+        <v>876</v>
+      </c>
+      <c r="B314" s="27">
+        <v>1018.17</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A315" t="s">
+        <v>877</v>
+      </c>
+      <c r="B315" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A316" t="s">
+        <v>878</v>
+      </c>
+      <c r="B316" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A317" t="s">
+        <v>879</v>
+      </c>
+      <c r="B317" s="27">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A318" t="s">
+        <v>880</v>
+      </c>
+      <c r="B318" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A319" t="s">
+        <v>881</v>
+      </c>
+      <c r="B319" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A320" t="s">
+        <v>882</v>
+      </c>
+      <c r="B320" s="27">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A321" t="s">
+        <v>883</v>
+      </c>
+      <c r="B321" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A322" t="s">
+        <v>884</v>
+      </c>
+      <c r="B322" s="27">
+        <v>1008.27</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A323" t="s">
+        <v>885</v>
+      </c>
+      <c r="B323" s="27">
+        <v>1153.26</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A324" t="s">
+        <v>886</v>
+      </c>
+      <c r="B324" s="27">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A325" t="s">
+        <v>887</v>
+      </c>
+      <c r="B325" s="27">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A326" t="s">
+        <v>888</v>
+      </c>
+      <c r="B326" s="27">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A327" t="s">
+        <v>889</v>
+      </c>
+      <c r="B327" s="27">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A328" t="s">
+        <v>890</v>
+      </c>
+      <c r="B328" s="27">
+        <v>1599.99</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A329" t="s">
+        <v>891</v>
+      </c>
+      <c r="B329" s="27">
+        <v>1699.99</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A330" t="s">
+        <v>892</v>
+      </c>
+      <c r="B330" s="27">
+        <v>1549.99</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A331" t="s">
+        <v>893</v>
+      </c>
+      <c r="B331" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A332" t="s">
+        <v>894</v>
+      </c>
+      <c r="B332" s="27">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="333" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A333" t="s">
+        <v>895</v>
+      </c>
+      <c r="B333" s="27">
+        <v>1699.99</v>
+      </c>
+    </row>
+    <row r="334" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A334" t="s">
+        <v>896</v>
+      </c>
+      <c r="B334" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A335" t="s">
+        <v>897</v>
+      </c>
+      <c r="B335" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="336" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A336" t="s">
+        <v>898</v>
+      </c>
+      <c r="B336" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="337" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A337" t="s">
+        <v>899</v>
+      </c>
+      <c r="B337" s="27">
+        <v>1799</v>
+      </c>
+    </row>
+    <row r="338" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A338" t="s">
+        <v>900</v>
+      </c>
+      <c r="B338" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="339" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A339" t="s">
+        <v>901</v>
+      </c>
+      <c r="B339" s="27">
+        <v>1599.99</v>
+      </c>
+    </row>
+    <row r="340" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A340" t="s">
+        <v>902</v>
+      </c>
+      <c r="B340" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="341" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A341" t="s">
+        <v>903</v>
+      </c>
+      <c r="B341" s="27">
+        <v>1543.19</v>
+      </c>
+    </row>
+    <row r="342" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A342" t="s">
+        <v>904</v>
+      </c>
+      <c r="B342" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="343" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A343" t="s">
+        <v>905</v>
+      </c>
+      <c r="B343" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="344" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A344" t="s">
+        <v>906</v>
+      </c>
+      <c r="B344" s="27">
+        <v>2299</v>
+      </c>
+    </row>
+    <row r="345" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A345" t="s">
+        <v>907</v>
+      </c>
+      <c r="B345" s="27">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="346" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A346" t="s">
+        <v>908</v>
+      </c>
+      <c r="B346" s="27">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="347" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A347" t="s">
+        <v>909</v>
+      </c>
+      <c r="B347" s="27">
+        <v>2407.31</v>
+      </c>
+    </row>
+    <row r="348" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A348" t="s">
+        <v>910</v>
+      </c>
+      <c r="B348" s="27">
+        <v>2699.99</v>
+      </c>
+    </row>
+    <row r="349" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A349" t="s">
+        <v>911</v>
+      </c>
+      <c r="B349" s="27">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="350" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A350" t="s">
+        <v>912</v>
+      </c>
+      <c r="B350" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="351" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A351" t="s">
+        <v>913</v>
+      </c>
+      <c r="B351" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="352" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A352" t="s">
+        <v>914</v>
+      </c>
+      <c r="B352" s="27">
+        <v>1166.6600000000001</v>
+      </c>
+    </row>
+    <row r="353" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A353" t="s">
+        <v>915</v>
+      </c>
+      <c r="B353" s="27">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="354" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A354" t="s">
+        <v>916</v>
+      </c>
+      <c r="B354" s="27">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="355" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A355" t="s">
+        <v>917</v>
+      </c>
+      <c r="B355" s="27">
+        <v>2999.99</v>
+      </c>
+    </row>
+    <row r="356" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A356" t="s">
+        <v>918</v>
+      </c>
+      <c r="B356" s="27">
+        <v>2166.66</v>
+      </c>
+    </row>
+    <row r="357" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A357" t="s">
+        <v>919</v>
+      </c>
+      <c r="B357" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="358" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A358" t="s">
+        <v>920</v>
+      </c>
+      <c r="B358" s="27">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="359" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A359" t="s">
+        <v>921</v>
+      </c>
+      <c r="B359" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="360" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A360" t="s">
+        <v>922</v>
+      </c>
+      <c r="B360" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="361" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A361" t="s">
+        <v>923</v>
+      </c>
+      <c r="B361" s="27">
+        <v>1799.99</v>
+      </c>
+    </row>
+    <row r="362" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A362" t="s">
+        <v>924</v>
+      </c>
+      <c r="B362" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="363" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A363" t="s">
+        <v>925</v>
+      </c>
+      <c r="B363" s="27">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="364" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A364" t="s">
+        <v>926</v>
+      </c>
+      <c r="B364" s="27">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="365" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A365" t="s">
+        <v>927</v>
+      </c>
+      <c r="B365" s="27">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="366" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A366" t="s">
+        <v>928</v>
+      </c>
+      <c r="B366" s="27">
+        <v>2499.9899999999998</v>
+      </c>
+    </row>
+    <row r="367" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A367" t="s">
+        <v>929</v>
+      </c>
+      <c r="B367" s="27">
+        <v>2699.99</v>
+      </c>
+    </row>
+    <row r="368" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A368" t="s">
+        <v>930</v>
+      </c>
+      <c r="B368" s="27">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="369" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A369" t="s">
+        <v>931</v>
+      </c>
+      <c r="B369" s="27">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="370" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A370" t="s">
+        <v>932</v>
+      </c>
+      <c r="B370" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="371" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A371" t="s">
+        <v>933</v>
+      </c>
+      <c r="B371" s="27">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="372" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A372" t="s">
+        <v>934</v>
+      </c>
+      <c r="B372" s="27">
+        <v>2399.9899999999998</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A373" t="s">
+        <v>935</v>
+      </c>
+      <c r="B373" s="27">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="374" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A374" t="s">
+        <v>936</v>
+      </c>
+      <c r="B374" s="27">
+        <v>1153.8399999999999</v>
+      </c>
+    </row>
+    <row r="375" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A375" t="s">
+        <v>937</v>
+      </c>
+      <c r="B375" s="27">
+        <v>1181.81</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A376" t="s">
+        <v>938</v>
+      </c>
+      <c r="B376" s="27">
+        <v>915.62</v>
+      </c>
+    </row>
+    <row r="377" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A377" t="s">
+        <v>939</v>
+      </c>
+      <c r="B377" s="27">
+        <v>1679.99</v>
+      </c>
+    </row>
+    <row r="378" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A378" t="s">
+        <v>940</v>
+      </c>
+      <c r="B378" s="27">
+        <v>1599.99</v>
+      </c>
+    </row>
+    <row r="379" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A379" t="s">
+        <v>941</v>
+      </c>
+      <c r="B379" s="27">
+        <v>1606.66</v>
+      </c>
+    </row>
+    <row r="380" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A380" t="s">
+        <v>942</v>
+      </c>
+      <c r="B380" s="27">
+        <v>1649.99</v>
+      </c>
+    </row>
+    <row r="381" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A381" t="s">
+        <v>943</v>
+      </c>
+      <c r="B381" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A382" t="s">
+        <v>944</v>
+      </c>
+      <c r="B382" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A383" t="s">
+        <v>945</v>
+      </c>
+      <c r="B383" s="27">
+        <v>1049.99</v>
+      </c>
+    </row>
+    <row r="384" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A384" t="s">
+        <v>946</v>
+      </c>
+      <c r="B384" s="27">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A385" t="s">
+        <v>947</v>
+      </c>
+      <c r="B385" s="27">
+        <v>1079.99</v>
+      </c>
+    </row>
+    <row r="386" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A386" t="s">
+        <v>948</v>
+      </c>
+      <c r="B386" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="387" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A387" t="s">
+        <v>949</v>
+      </c>
+      <c r="B387" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="388" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A388" t="s">
+        <v>950</v>
+      </c>
+      <c r="B388" s="27">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A389" t="s">
+        <v>951</v>
+      </c>
+      <c r="B389" s="27">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="390" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A390" t="s">
+        <v>952</v>
+      </c>
+      <c r="B390" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A391" t="s">
+        <v>953</v>
+      </c>
+      <c r="B391" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A392" t="s">
+        <v>954</v>
+      </c>
+      <c r="B392" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="393" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A393" t="s">
+        <v>955</v>
+      </c>
+      <c r="B393" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="394" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A394" t="s">
+        <v>956</v>
+      </c>
+      <c r="B394" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="395" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A395" t="s">
+        <v>957</v>
+      </c>
+      <c r="B395" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="396" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A396" t="s">
+        <v>958</v>
+      </c>
+      <c r="B396" s="27">
+        <v>2399.9899999999998</v>
+      </c>
+    </row>
+    <row r="397" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A397" t="s">
+        <v>959</v>
+      </c>
+      <c r="B397" s="27">
+        <v>2399.9899999999998</v>
+      </c>
+    </row>
+    <row r="398" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A398" t="s">
+        <v>960</v>
+      </c>
+      <c r="B398" s="27">
+        <v>2799.99</v>
+      </c>
+    </row>
+    <row r="399" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A399" t="s">
+        <v>961</v>
+      </c>
+      <c r="B399" s="27">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="400" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A400" t="s">
+        <v>962</v>
+      </c>
+      <c r="B400" s="27">
+        <v>2199.9899999999998</v>
+      </c>
+    </row>
+    <row r="401" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A401" t="s">
+        <v>963</v>
+      </c>
+      <c r="B401" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="402" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A402" t="s">
+        <v>964</v>
+      </c>
+      <c r="B402" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="403" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A403" t="s">
+        <v>965</v>
+      </c>
+      <c r="B403" s="27">
+        <v>1299.99</v>
+      </c>
+    </row>
+    <row r="404" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A404" t="s">
+        <v>966</v>
+      </c>
+      <c r="B404" s="27">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="405" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A405" t="s">
+        <v>967</v>
+      </c>
+      <c r="B405" s="27">
+        <v>799.99</v>
+      </c>
+    </row>
+    <row r="406" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A406" t="s">
+        <v>968</v>
+      </c>
+      <c r="B406" s="27">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="407" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A407" t="s">
+        <v>969</v>
+      </c>
+      <c r="B407" s="27">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="408" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A408" t="s">
+        <v>970</v>
+      </c>
+      <c r="B408" s="27">
+        <v>1199.99</v>
+      </c>
+    </row>
+    <row r="409" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A409" t="s">
+        <v>971</v>
+      </c>
+      <c r="B409" s="27">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="410" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A410" t="s">
+        <v>972</v>
+      </c>
+      <c r="B410" s="27">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="411" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A411" t="s">
+        <v>973</v>
+      </c>
+      <c r="B411" s="27">
+        <v>1999.99</v>
+      </c>
+    </row>
+    <row r="412" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A412" t="s">
+        <v>974</v>
+      </c>
+      <c r="B412" s="27">
+        <v>1499.99</v>
+      </c>
+    </row>
+    <row r="413" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A413" t="s">
+        <v>975</v>
+      </c>
+      <c r="B413" s="27">
+        <v>1599.99</v>
+      </c>
+    </row>
+    <row r="414" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A414" t="s">
+        <v>976</v>
+      </c>
+      <c r="B414" s="27">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="415" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A415" t="s">
+        <v>977</v>
+      </c>
+      <c r="B415" s="27">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="416" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A416" t="s">
+        <v>978</v>
+      </c>
+      <c r="B416" s="27">
+        <v>300</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40DD5561-C71A-4E3E-8C3F-36B212A5A12C}">
   <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2987,7 +7600,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4489C6B-D1C2-415E-B0B3-CC749A9F03E5}">
   <dimension ref="A1:C234"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5576,7 +10189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{206F00A0-332C-413C-836F-690379DEF35A}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5649,7 +10262,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{525F9421-13B4-413F-B405-CE8C1993584F}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>